<commit_message>
live update 19:17:50 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-lavked-g2a-2026-04-02_20260402_191249.xlsx
+++ b/data/live_logs/live_cs2-lavked-g2a-2026-04-02_20260402_191249.xlsx
@@ -34,7 +34,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,12 @@
         <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -66,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -75,6 +81,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AD5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -737,6 +745,336 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>19:13:23</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>23</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>11-12</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.1815</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.5907</v>
+      </c>
+      <c r="J3" t="n">
+        <v>7500</v>
+      </c>
+      <c r="K3" t="n">
+        <v>8400</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>73</v>
+      </c>
+      <c r="O3" t="n">
+        <v>79</v>
+      </c>
+      <c r="P3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>14</v>
+      </c>
+      <c r="R3" t="n">
+        <v>8</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="V3" t="n">
+        <v>6017.3868</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>0.2207396748661995</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>MAP2:Lavked@0.497x181; WINNER:G2 Ares@0.340x209</t>
+        </is>
+      </c>
+      <c r="Z3" t="n">
+        <v>96800</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>99800.91</v>
+      </c>
+      <c r="AB3" s="4" t="inlineStr">
+        <is>
+          <t>BUY WINNER G2 Ares $71@0.340  SELL MAP1 G2 Ares P/L:$+96800.00</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>19:15:52</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>12-12</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.1815</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.5907</v>
+      </c>
+      <c r="J4" t="n">
+        <v>7500</v>
+      </c>
+      <c r="K4" t="n">
+        <v>8400</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>73</v>
+      </c>
+      <c r="O4" t="n">
+        <v>79</v>
+      </c>
+      <c r="P4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>14</v>
+      </c>
+      <c r="R4" t="n">
+        <v>8</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="V4" t="n">
+        <v>6017.3868</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>0.8466543736457824</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>MAP2:Lavked@0.497x181; WINNER:G2 Ares@0.340x209; MAP1:G2 Ares@0.001x83904</t>
+        </is>
+      </c>
+      <c r="Z4" t="n">
+        <v>96800</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>53.26</v>
+      </c>
+      <c r="AB4" s="4" t="inlineStr">
+        <is>
+          <t>BUY MAP1 G2 Ares $84@0.001</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>19:16:04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>24</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>12-12</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0.2944</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.6472</v>
+      </c>
+      <c r="J5" t="n">
+        <v>9750</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1700</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>77</v>
+      </c>
+      <c r="O5" t="n">
+        <v>80</v>
+      </c>
+      <c r="P5" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>14</v>
+      </c>
+      <c r="R5" t="n">
+        <v>9</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="V5" t="n">
+        <v>6017.3868</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z5" t="n">
+        <v>178067.42</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>83796.24000000001</v>
+      </c>
+      <c r="AB5" s="4" t="inlineStr">
+        <is>
+          <t>SELL WINNER G2 Ares P/L:$+70.96  SELL MAP1 G2 Ares P/L:$+81219.46  FORCE-EXIT MAP2 Lavked P/L:$-23.00</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -748,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -756,14 +1094,14 @@
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -933,6 +1271,312 @@
       </c>
       <c r="M3" s="7" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>19:13:23</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>23</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>208.6941176470588</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>0.5907396748661995</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>0.2207396748661995</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>19:13:23</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>23</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>0.8776543736457825</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>-0.1213456263542175</v>
+      </c>
+      <c r="M5" s="8" t="n">
+        <v>96800</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>19:15:52</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>23</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>83904.39999999999</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0.8776543736457825</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>0.8466543736457824</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>19:16:04</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>24</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>208.6941176470588</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0.6472128629684448</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>-0.06278713703155514</v>
+      </c>
+      <c r="M7" s="8" t="n">
+        <v>70.95599999999997</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>19:16:04</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>24</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>83904.39999999999</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>0.8776543736457825</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>-0.1213456263542175</v>
+      </c>
+      <c r="M8" s="8" t="n">
+        <v>81219.4592</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>19:16:04</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MAP2</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>FORCE-EXIT</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Lavked</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>181.0865191146881</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>0.7055742740631104</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.3055742740631103</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>-22.99798792756539</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
live update 19:22:55 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-lavked-g2a-2026-04-02_20260402_191249.xlsx
+++ b/data/live_logs/live_cs2-lavked-g2a-2026-04-02_20260402_191249.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD5"/>
+  <dimension ref="A1:AD6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -474,7 +474,7 @@
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="23" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="21" customWidth="1" min="24" max="24"/>
     <col width="30" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -1070,6 +1070,120 @@
         </is>
       </c>
       <c r="AD5" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>19:21:19</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>13-12</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.6713</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.8357</v>
+      </c>
+      <c r="J6" t="n">
+        <v>11900</v>
+      </c>
+      <c r="K6" t="n">
+        <v>6500</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O6" t="n">
+        <v>81</v>
+      </c>
+      <c r="P6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R6" t="n">
+        <v>10</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="V6" t="n">
+        <v>6017.3868</v>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>0.7256744647026062</v>
+      </c>
+      <c r="X6" s="3" t="n">
+        <v>0.4973489294052124</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>WINNER:G2 Ares@0.080x1250; MAP1:G2 Ares@0.001x90000; MAP2:G2 Ares@0.144x562</t>
+        </is>
+      </c>
+      <c r="Z6" t="n">
+        <v>178067.42</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="4" t="inlineStr">
+        <is>
+          <t>BUY WINNER G2 Ares $100@0.080  BUY MAP1 G2 Ares $90@0.001  BUY MAP2 G2 Ares $81@0.144</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
         <is>
           <t>SPARTA</t>
         </is>
@@ -1086,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1579,6 +1693,159 @@
         <v>-22.99798792756539</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>19:21:19</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>25</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>1250</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>0.8356744647026062</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>0.7256744647026062</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>19:21:19</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>25</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>90000</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>0.8776543736457825</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>0.8466543736457824</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>19:21:19</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>25</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>MAP2</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>562.5</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>0.6713489294052124</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>0.4973489294052124</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>